<commit_message>
Reorganizing the data so we can have a filtered pipeline
</commit_message>
<xml_diff>
--- a/data/Site_S_USGS_Thesis_matchguide.xlsx
+++ b/data/Site_S_USGS_Thesis_matchguide.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mailsfsu-my.sharepoint.com/personal/924318106_sfsu_edu/Documents/ProjectData/GitHub/DepositionSFB/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="8_{35722EBA-5731-4EBC-80FF-45ED5270C9F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{87DBE76E-3F80-405C-B71F-7D5DCF08EB0F}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="8_{35722EBA-5731-4EBC-80FF-45ED5270C9F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4F0FE515-1EB3-40CF-82EE-0EED6D5722A2}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="3348" yWindow="3348" windowWidth="17280" windowHeight="9420" xr2:uid="{03EE2BC8-78E9-4368-8265-B212D255FCBD}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{03EE2BC8-78E9-4368-8265-B212D255FCBD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="9">
   <si>
     <t>Thesis Site S Locations</t>
   </si>
@@ -63,6 +63,9 @@
   </si>
   <si>
     <t>USGS Site C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   </t>
   </si>
 </sst>
 </file>
@@ -445,7 +448,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4D13550-AC90-4C24-90CE-553E0BAF5F42}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
@@ -690,6 +693,11 @@
         <v>5</v>
       </c>
     </row>
+    <row r="17" spans="10:10" x14ac:dyDescent="0.3">
+      <c r="J17" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>